<commit_message>
Show conditional formatting in .xls and .ods sheets
The rule engine is now shared by all three spreadsheet readers. .ods files use LibreOffice's conditional formats (value and text rules, colour scales, data bars, icon sets); .xls files use their CF value rules. Formula rules are counted in a notice.
</commit_message>
<xml_diff>
--- a/tests/corpus/xlsx/conditional.xlsx
+++ b/tests/corpus/xlsx/conditional.xlsx
@@ -613,8 +613,8 @@
         <color rgb="FF638EC6"/>
       </dataBar>
       <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{87C45FDB-1BFD-4746-8D0C-7AE1E23C8C4D}</x14:id>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{00000000-0000-4000-8000-000000000001}">
+          <x14:id>{00000000-0000-4000-8000-000000000001}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -641,10 +641,10 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{00000000-0000-4000-8000-000000000001}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{87C45FDB-1BFD-4746-8D0C-7AE1E23C8C4D}">
+          <x14:cfRule type="dataBar" id="{00000000-0000-4000-8000-000000000001}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>

</xml_diff>